<commit_message>
Add new database (PointFinder)
</commit_message>
<xml_diff>
--- a/data/database_status.xlsx
+++ b/data/database_status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uqlngo2\Documents\GitHub\RIFR_Map\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB140CD1-32E8-4796-8FE6-19D69FA99EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3682C51F-D5F8-4C68-9B99-A797638EE788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="11500" xr2:uid="{9BBD2626-AADE-4B89-8BD3-2FC849FF55ED}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{9BBD2626-AADE-4B89-8BD3-2FC849FF55ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>Database</t>
   </si>
@@ -117,6 +117,9 @@
   </si>
   <si>
     <t>https://www.nature.com/articles/s41598-021-91456-0</t>
+  </si>
+  <si>
+    <t>PointFinder</t>
   </si>
 </sst>
 </file>
@@ -488,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EABEBCF3-8632-4D7F-A7B9-07630C6D851C}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="51.36328125" bestFit="1" customWidth="1"/>
@@ -595,6 +598,14 @@
         <v>18</v>
       </c>
     </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>